<commit_message>
Update public opportunity workbook sample
</commit_message>
<xml_diff>
--- a/public/public-opportunity-desk/Grant-Admin-Support-Sample-Workbook-2026-05-14.xlsx
+++ b/public/public-opportunity-desk/Grant-Admin-Support-Sample-Workbook-2026-05-14.xlsx
@@ -12,8 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Document Checklist" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Log" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFR Evidence Map" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Questions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Change Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approval Dependencies" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closeout Tracker" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation Questions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -234,8 +237,51 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="WorkbookChecks" displayName="WorkbookChecks" ref="A3:D11" headerRowCount="1">
-  <autoFilter ref="A3:D11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="CloseoutSubmissionTracker" displayName="CloseoutSubmissionTracker" ref="A3:H8" headerRowCount="1">
+  <autoFilter ref="A3:H8"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Closeout ID"/>
+    <tableColumn id="2" name="Phase"/>
+    <tableColumn id="3" name="Required Evidence"/>
+    <tableColumn id="4" name="Source Anchor"/>
+    <tableColumn id="5" name="Support Task"/>
+    <tableColumn id="6" name="Owner"/>
+    <tableColumn id="7" name="Status"/>
+    <tableColumn id="8" name="Boundary"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="ValidationQuestions" displayName="ValidationQuestions" ref="A3:E8" headerRowCount="1">
+  <autoFilter ref="A3:E8"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Question ID"/>
+    <tableColumn id="2" name="Question"/>
+    <tableColumn id="3" name="Reviewer Response"/>
+    <tableColumn id="4" name="Score"/>
+    <tableColumn id="5" name="Follow-Up Action"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="AcceptanceCriteria" displayName="AcceptanceCriteria" ref="A12:C17" headerRowCount="1">
+  <autoFilter ref="A12:C17"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Acceptance Criteria"/>
+    <tableColumn id="2" name="Met?"/>
+    <tableColumn id="3" name="Evidence"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="WorkbookChecks" displayName="WorkbookChecks" ref="A3:D14" headerRowCount="1">
+  <autoFilter ref="A3:D14"/>
   <tableColumns count="4">
     <tableColumn id="1" name="Check"/>
     <tableColumn id="2" name="Formula / Value"/>
@@ -247,8 +293,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="WorkbookSections" displayName="WorkbookSections" ref="D4:E10" headerRowCount="1">
-  <autoFilter ref="D4:E10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="WorkbookSections" displayName="WorkbookSections" ref="D4:E13" headerRowCount="1">
+  <autoFilter ref="D4:E13"/>
   <tableColumns count="2">
     <tableColumn id="4" name="Workbook Sections"/>
     <tableColumn id="5" name="Purpose"/>
@@ -337,26 +383,34 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ValidationQuestions" displayName="ValidationQuestions" ref="A3:E8" headerRowCount="1">
-  <autoFilter ref="A3:E8"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Question ID"/>
-    <tableColumn id="2" name="Question"/>
-    <tableColumn id="3" name="Reviewer Response"/>
-    <tableColumn id="4" name="Score"/>
-    <tableColumn id="5" name="Follow-Up Action"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="SourceChangeLog" displayName="SourceChangeLog" ref="A3:H7" headerRowCount="1">
+  <autoFilter ref="A3:H7"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Change ID"/>
+    <tableColumn id="2" name="Source"/>
+    <tableColumn id="3" name="Change Type"/>
+    <tableColumn id="4" name="Public-Source Evidence"/>
+    <tableColumn id="5" name="Support Action"/>
+    <tableColumn id="6" name="Boundary"/>
+    <tableColumn id="7" name="Reviewer Status"/>
+    <tableColumn id="8" name="Reviewer Notes"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AcceptanceCriteria" displayName="AcceptanceCriteria" ref="A12:C17" headerRowCount="1">
-  <autoFilter ref="A12:C17"/>
-  <tableColumns count="3">
-    <tableColumn id="1" name="Acceptance Criteria"/>
-    <tableColumn id="2" name="Met?"/>
-    <tableColumn id="3" name="Evidence"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="ApprovalDependencyLog" displayName="ApprovalDependencyLog" ref="A3:H7" headerRowCount="1">
+  <autoFilter ref="A3:H7"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="Dependency ID"/>
+    <tableColumn id="2" name="Dependency"/>
+    <tableColumn id="3" name="Source Anchor"/>
+    <tableColumn id="4" name="Why It Matters"/>
+    <tableColumn id="5" name="Andy Support Output"/>
+    <tableColumn id="6" name="Required Owner"/>
+    <tableColumn id="7" name="Status"/>
+    <tableColumn id="8" name="Boundary"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -843,12 +897,12 @@
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Validation Questions</t>
+          <t>Source Change Log</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Capture whether a qualified reviewer thinks the support packet is useful, risky, generic, or worth narrowing.</t>
+          <t>Track public addenda, package changes, guidance refreshes, and workbook sections affected by source changes.</t>
         </is>
       </c>
       <c r="F9" s="4" t="n"/>
@@ -869,12 +923,12 @@
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Checks</t>
+          <t>Approval Dependencies</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Audit workbook counts, scope gates, and proof status.</t>
+          <t>Keep FloridaCommerce, HUD/CDBG, official submission, and validation-gate dependencies explicit.</t>
         </is>
       </c>
       <c r="F10" s="4" t="n"/>
@@ -893,8 +947,16 @@
         </is>
       </c>
       <c r="C11" s="4" t="n"/>
-      <c r="D11" s="4" t="n"/>
-      <c r="E11" s="4" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Closeout Tracker</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Map annual submissions, final closeout, retention, monitoring, and public-records handoff evidence.</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
@@ -903,8 +965,16 @@
       <c r="A12" s="4" t="n"/>
       <c r="B12" s="4" t="n"/>
       <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Validation Questions</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Capture whether a qualified reviewer thinks the support packet is useful, risky, generic, or worth narrowing.</t>
+        </is>
+      </c>
       <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
@@ -913,8 +983,16 @@
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="n"/>
       <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Checks</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Audit workbook counts, scope gates, and proof status.</t>
+        </is>
+      </c>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
@@ -1110,6 +1188,347 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Workbook Checks</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>These checks support artifact review only; they do not prove income.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Formula / Value</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
+      <c r="G3" s="4" t="n"/>
+      <c r="H3" s="4" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Proof status</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+      <c r="D4" s="4">
+        <f>IF(B4=C4,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tracker rows</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>COUNTA('Reimbursement Tracker'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4">
+        <f>IF(B5=C5,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Checklist rows</t>
+        </is>
+      </c>
+      <c r="B6" s="4">
+        <f>COUNTA('Document Checklist'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4">
+        <f>IF(B6=C6,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Risk rows</t>
+        </is>
+      </c>
+      <c r="B7" s="4">
+        <f>COUNTA('Risk Log'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4">
+        <f>IF(B7=C7,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="4" t="n"/>
+      <c r="H7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Evidence map rows</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>COUNTA('CFR Evidence Map'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4">
+        <f>IF(B8=C8,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Source change rows</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>COUNTA('Source Change Log'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="4">
+        <f>IF(B9=C9,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Approval dependency rows</t>
+        </is>
+      </c>
+      <c r="B10" s="4">
+        <f>COUNTA('Approval Dependencies'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D10" s="4">
+        <f>IF(B10=C10,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Closeout rows</t>
+        </is>
+      </c>
+      <c r="B11" s="4">
+        <f>COUNTA('Closeout Tracker'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4">
+        <f>IF(B11=C11,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Validation questions</t>
+        </is>
+      </c>
+      <c r="B12" s="4">
+        <f>COUNTA('Validation Questions'!A4:A200)</f>
+        <v/>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="4">
+        <f>IF(B12=C12,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>No official submission</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D13" s="4">
+        <f>IF(B13=C13,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>No payment request</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D14" s="4">
+        <f>IF(B14=C14,"OK","Review")</f>
+        <v/>
+      </c>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="n"/>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D4:D40">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$D4="Review"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>$D4="OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2231,6 +2650,872 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source Change Log</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Track public-source changes before a reviewer relies on the workbook.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Change ID</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Change Type</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Public-Source Evidence</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Support Action</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer Status</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Reviewer Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>chg-001</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>City of Avon Park RFP #26-05 public RFP page</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>addendum and public-source update tracking</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Public RFP pages and supporting documents can change through addenda before submission deadlines.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Track last public-source check, addendum number if visible, changed section, and whether the workbook needs updates.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Do not contact the agency, register in a portal, or submit questions without separate approval.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>chg-002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>JEA Grant Administrator for Normandy Village Utility solicitation</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>package-controlled scope detail</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>The JEA page points bidders to the solicitation package for minimum qualifications, forms, and details.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Keep a placeholder for package-controlled requirements and prevent unsupported assumptions in the workbook.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>No portal credentials or official bid package action.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>chg-003</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>FloridaCommerce Infrastructure Repair Program</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>program guidance update</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>State program pages can update program notices, eligible activities, deadlines, or implementation guidance.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Record program-source URL, check date, changed guidance area, and affected workbook sections.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>No eligibility decision or compliance interpretation.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>chg-004</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>HUD CDBG-DR FAQs and 2 CFR Part 200</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>reference-source refresh</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Federal guidance and regulatory references anchor the evidence categories used by the sample.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Track whether source references were rechecked before a reviewer relies on the workbook.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>No legal advice, procurement advice, or compliance certification.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G4:G200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$G4="blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="G4:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"sample_not_started,needs_review,complete,blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Approval Dependencies</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Approval dependency tracker. This sheet does not represent approvals obtained.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Dependency ID</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Dependency</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Source Anchor</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Why It Matters</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Andy Support Output</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Required Owner</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>dep-001</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>FloridaCommerce approval or program-owner approval condition</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>City of Avon Park RFP #26-05 and FloridaCommerce CDBG-DR program surface</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>A selected grant-admin scope or contract can remain contingent on the responsible program owner's approval.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>List approval checkpoints, owner, evidence needed, and open status.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>qualified grant administrator or municipal program owner</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Do not represent that approval has been obtained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>dep-002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>HUD CDBG-DR and 2 CFR evidence review</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>HUD CDBG-DR FAQs and 2 CFR Part 200</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>The support packet must stay behind a qualified reviewer for procurement, allowability, audit, and reporting judgments.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Organize evidence categories and missing-document flags.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>qualified grant administrator, counsel, procurement owner, or finance owner</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>needs_review</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>No compliance opinion or allowability certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>dep-003</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Official submission owner</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>JEA solicitation package boundary and public procurement norms</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Only authorized parties should submit, certify, or approve official grant or procurement records.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Prepare internal readiness views and reviewer notes.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>authorized public owner or prime grant administrator</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>blocked_until_approved</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>No official submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>dep-004</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>No-charge validation gate</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>route decision matrix</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>The lane only advances if a qualified reviewer confirms the artifact is useful and safely bounded.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Show one support-only workbook and record specific validation feedback.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Andy after explicit approval phrase</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>blocked_until_approved</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>No outreach without the exact approval phrase.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G4:G200">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>$G4="blocked_until_approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="G4:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"sample_not_started,needs_review,complete,blocked_until_approved"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Closeout Tracker</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Support-only closeout evidence map for qualified reviewer use.</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Closeout ID</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Required Evidence</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Source Anchor</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Support Task</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>close-001</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>annual or periodic submissions</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>reporting calendar, responsible owner, supporting source-document index, unresolved issue log</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>City of Avon Park RFP #26-05 references grant administration support through program reporting and submissions.</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Create a non-official calendar and evidence-readiness checklist for reviewer use.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>qualified grant administrator or municipal program owner</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>No official reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>close-002</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>final closeout package</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>final reimbursement index, budget-to-actual reconciliation, procurement file index, payment proof, outstanding conditions</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Avon Park CDBG-DR RFP and 2 CFR audit/readiness source categories</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Track closeout packet completeness and unresolved evidence gaps.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>qualified grant administrator</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>No certification of closeout sufficiency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>close-003</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>record retention and audit handoff</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>retention index, file location, responsible custodian, audit-reference notes</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2 CFR Part 200 includes audit requirements and record-support expectations.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Prepare an index of records and missing file flags for the official owner.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>finance owner or records custodian</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Do not set official retention policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>close-004</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>monitoring or corrective-action follow-up</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>monitoring findings, corrective action owner, due dates, resolution evidence</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>CDBG-DR program management work commonly includes monitoring and closeout support.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Track open findings and evidence links without drafting official responses.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>qualified grant administrator or public owner</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>No official agency response.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>close-005</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>public records handoff</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>public-records file index, excluded sensitive fields note, access owner, file location</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Florida public-sector grant work can be subject to public-records handling and later review.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Organize a public-records-safe handoff index and mark items requiring owner review.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>public records custodian or municipal owner</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>sample_not_started</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>No public-records legal determination.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G4:G200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$G4="blocked"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="G4:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"sample_not_started,needs_review,complete,blocked"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2531,279 +3816,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Workbook Checks</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>These checks support artifact review only; they do not prove income.</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Formula / Value</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Proof status</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="D4" s="4">
-        <f>IF(B4=C4,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Tracker rows</t>
-        </is>
-      </c>
-      <c r="B5" s="4">
-        <f>COUNTA('Reimbursement Tracker'!A4:A200)</f>
-        <v/>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D5" s="4">
-        <f>IF(B5=C5,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Checklist rows</t>
-        </is>
-      </c>
-      <c r="B6" s="4">
-        <f>COUNTA('Document Checklist'!A4:A200)</f>
-        <v/>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" s="4">
-        <f>IF(B6=C6,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Risk rows</t>
-        </is>
-      </c>
-      <c r="B7" s="4">
-        <f>COUNTA('Risk Log'!A4:A200)</f>
-        <v/>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="4">
-        <f>IF(B7=C7,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Evidence map rows</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>COUNTA('CFR Evidence Map'!A4:A200)</f>
-        <v/>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="4">
-        <f>IF(B8=C8,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Validation questions</t>
-        </is>
-      </c>
-      <c r="B9" s="4">
-        <f>COUNTA('Validation Questions'!A4:A200)</f>
-        <v/>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="4">
-        <f>IF(B9=C9,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>No official submission</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D10" s="4">
-        <f>IF(B10=C10,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>No payment request</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D11" s="4">
-        <f>IF(B11=C11,"OK","Review")</f>
-        <v/>
-      </c>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <conditionalFormatting sqref="D4:D40">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$D4="Review"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="2">
-      <formula>$D4="OK"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup fitToHeight="0" fitToWidth="1"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>